<commit_message>
chore(trackers): sync branch to main + regenerate reconcile snapshot
Merge origin/main (resolves verify-branch-fresh behind-count) + regen
block-reconciliation-data.json against current tree. Counts stable:
1186 total / 504 audit-note / 34 to build.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-19.xlsx
+++ b/docs/trackers/exports/IH35-TMS-BLOCK-RECONCILIATION-2026-07-19.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7136" uniqueCount="1716">
   <si>
-    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-19 (verified vs origin/main + 2621 merged PRs)</t>
+    <t>IH35-TMS — EVERY BLOCK, BUILT vs PENDING — 2026-07-19 (verified vs origin/main + 2630 merged PRs)</t>
   </si>
   <si>
     <t>DONE = verified on main (branch merged or files present) · NEEDS-VERIFY = weak signal, not trusted until GUARD confirms · PENDING = needs build · PENDING (GATED) = financial/locked, needs Jorge's gate first</t>
@@ -29477,7 +29477,7 @@
         <v>1714</v>
       </c>
       <c r="B10">
-        <v>2621</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -29485,7 +29485,7 @@
         <v>1715</v>
       </c>
       <c r="B11">
-        <v>9929</v>
+        <v>9947</v>
       </c>
     </row>
   </sheetData>

</xml_diff>